<commit_message>
Tablas_Stock vigente - Sep-2026
</commit_message>
<xml_diff>
--- a/Tablas/Tablas_Stock.xlsx
+++ b/Tablas/Tablas_Stock.xlsx
@@ -458,7 +458,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Demanda del vecino 3.559 casos: sube 20% vs julio pero sigue 22% por debajo del promedio 2026 (4.580) y es el 2do mes más bajo del año. La carga baja 30% desde el pico de abril (5.074): mejora sostenida. Excepción: CALLES Y VEREDAS 405, máximo de toda la serie y en alza todo el año.</t>
+          <t>Demanda del vecino 4.073 casos: +15% vs agosto y +34% vs Sep-2025, segundo mes de suba desde el piso de julio. Sigue 11% debajo del promedio ene-jun (4.578). Suben Escombros (605, maximo de la serie), poda domiciliaria y cordon; baja luminaria apagada (-95).</t>
         </is>
       </c>
     </row>
@@ -470,7 +470,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Cierre global 73% (-3pp vs julio). ALUMBRADO 89%, RESIDUOS 86% y CTRL ACTIVIDADES 78% lideran. Crítico: CALLES 20% (sexto mes en zona crítica) y ARBOLADO cae a 49%. Cancelado sobre cerrados: ninguna área supera el 10% (máximo TRÁNSITO y ARBOLADO 8%).</t>
+          <t>Cierre global 72% (-1pp vs agosto). RESIDUOS y CTRL ACTIVIDADES 88%, ALUMBRADO 83% lideran. Critico: CALLES 15% (septimo mes bajo 50%) y CTRL ESPACIO cae a 39% por Cable cortado (117 casos, 1 cierre). Cancelado sobre cerrados: ARBOLADO 11%, CALLES 7%, TRANSITO 3%.</t>
         </is>
       </c>
     </row>
@@ -482,7 +482,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>SLA global 51% (+7pp vs julio). ARBOLADO 77% y CTRL ESPACIO 76% lideran; ALUMBRADO 62%. Más bajos: TRÁNSITO y CALLES 31%. Promedio 5 días para cerrados; CALLES sube a 9 días.</t>
+          <t>SLA global 55% (+4pp vs agosto). CTRL ESPACIO 86% y ARBOLADO 81% lideran; ALUMBRADO 75%. Mas bajos: CALLES 28% y RESIDUOS 47% (escombros y poda cierran en 4 dias con plazo 2). Promedio 4 dias; CALLES sube a 10. Umbrales nuevos desde septiembre: serie no comparable.</t>
         </is>
       </c>
     </row>
@@ -494,7 +494,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Satisfacción global 69% (+2pp vs julio). 526 respuestas, tasa 14.8% del total (18% s/incidentes con email). RESIDUOS 73%, ALUMBRADO 72% y TRÁNSITO 71%; CTRL ACTIVIDADES 33%. CALLES y TRÁNSITO con muestra insuficiente.</t>
+          <t>Satisfaccion global 69% (+0pp vs agosto). 681 respuestas, tasa 23% sobre cumplidos. ALUMBRADO 78%, RESIDUOS y TRANSITO 73%; ARBOLADO 10% (2 de 20) es la peor del municipio y CTRL ACTIVIDADES 31% mantiene la brecha con su cierre. CALLES y TRANSITO con muestra insuficiente.</t>
         </is>
       </c>
     </row>
@@ -536,7 +536,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>El área que mejor responde: cierra el 89% de sus 565 reclamos en 4 días promedio. Siete de cada diez son luminarias apagadas de noche (398 casos), una suba que se repite cada invierno. La mitad de su carga la detecta el propio municipio, no el vecino.</t>
+          <t>Baja 17% tras el pico de agosto y vuelve al nivel de hace un año (468). Cierra el 83% en 3 días con la mejor satisfacción del municipio (78%). Cuando una luminaria apagada se pasa del plazo de 3 días tarda casi 5. La mitad de su carga la detecta el propio municipio.</t>
         </is>
       </c>
     </row>
@@ -548,7 +548,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Más que duplicó su demanda (98 casos) y el cierre cayó a 49%: resuelve rápido lo que atiende, pero deja la mitad sin cerrar. El corte de césped arrancó un mes antes que el año pasado y ya acumula 23 reclamos con apenas 17% de cierre.</t>
+          <t>Sube 66% (131 casos) y recupera el cierre (56%), pero el vecino no lo percibe: 10% de satisfacción, la peor del municipio, con 12 de 16 respuestas insatisfechas en intervenciones de arbolado. Árbol obstruye luminaria pasa de 11 a 38 casos con 11% de cierre.</t>
         </is>
       </c>
     </row>
@@ -560,7 +560,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>El cuadro más crítico del municipio: recibe el máximo histórico de reclamos (405, el doble que en enero) y cierra uno de cada cinco, con 9 días promedio. Los baches de asfalto (178 casos) marcan un deterioro real del pavimento, no estacional.</t>
+          <t>El cuadro más crítico, y empeora: máximo histórico de 470 reclamos (+53% interanual), cierre que cae a 15% y 10 días promedio. El cordón se dispara a 111 casos con 5% de cierre y los baches de asfalto (166) cierran uno de cada cuatro. Séptimo mes en zona crítica.</t>
         </is>
       </c>
     </row>
@@ -572,7 +572,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Cierra bien —78% de 101 reclamos— pero el vecino no lo percibe así: la satisfacción es del 33%, la más baja del municipio. Predominan las denuncias por falta de habilitación comercial (37 casos), donde cerrar el expediente no siempre resuelve el problema.</t>
+          <t>Demanda en baja (95 casos, -14%) y cierre alto (88%, sin cancelaciones), pero la satisfacción sigue en 31%: ruidos molestos (29 casos) y plagas concentran las respuestas insatisfechas. Cerrar el expediente no resuelve lo que el vecino denuncia.</t>
         </is>
       </c>
     </row>
@@ -584,7 +584,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Demanda en baja sostenida (275 casos, desde 393 en enero), pero con el cierre partido en dos: resuelve el 100% de las desratizaciones y apenas el 12% de los cables cortados y el 22% de los postes en mal estado.</t>
+          <t>La demanda sube 20% (318) y el cierre se desploma a 39% por un solo tipo: cable cortado, 117 casos (el triple que hace un año) con un solo cierre. Sin ese tipo el área cerraría el 62%. Roedores (83) sigue cerrando el 92% en poco más de un día y lidera el SLA (86%).</t>
         </is>
       </c>
     </row>
@@ -596,7 +596,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Concentra casi la mitad de la demanda del municipio (1.657 casos) y la viene reduciendo con fuerza: 45% menos que en enero. Cierra el 86% en 5 días. El grueso son retiros a domicilio de escombros, restos de poda y objetos en desuso.</t>
+          <t>Arranca la temporada alta: 2.076 casos (+24%, +40% interanual). Escombros marca su máximo (605) y la poda domiciliaria sube a 423. Cierra el 88% en 6 días con 73% de satisfacción, pero solo la mitad dentro del plazo de 2 días. El barrido (179) cerró su ciclo anómalo.</t>
         </is>
       </c>
     </row>
@@ -608,7 +608,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Demanda estable (458 casos) y cierre del 70%, pero lento: solo el 31% se resuelve dentro del plazo comprometido. Tres de cada cuatro reclamos son vehículos abandonados (346 casos). La satisfacción del 71% surge de apenas 17 respuestas.</t>
+          <t>Demanda estable en 515 (+13%), cierre del 72% y SLA que mejora a 59%. Los vehículos abandonados (392, tres de cada cuatro reclamos) cierran el 82% pero suman 10 cancelaciones; los semáforos (77) cierran la mitad y tardan 9 días cuando se pasan. 73% de satisfacción, 22 respuestas.</t>
         </is>
       </c>
     </row>
@@ -623,13 +623,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="38" customWidth="1" min="3" max="3"/>
-    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="90" customWidth="1" min="6" max="6"/>
   </cols>
@@ -674,7 +674,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Jul-2026</t>
+          <t>Ago-2026</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -684,81 +684,81 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
+          <t>Cierre bajo (area)</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>49%-&gt;56%</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Cierre del area sube de 49% a 56% (Ago-2026 a Sep-2026). Sale de la zona critica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>PERSISTE</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Mar-2026</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Calles y Veredas</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Cierre colapsado</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>20%-&gt;15%</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Cierre del area 20%-&gt;15% (Ago-2026 a Sep-2026), séptimo mes en zona crítica. Cancelado 7% sobre cerrados; 399 casos sin cerrar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>PERSISTE</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Ago-2026</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Calles y Veredas</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
           <t>Dias promedio alto</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>4 dias</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Tiempo promedio de resolucion baja a 4 dias en Ago-2026 (tablero). Vuelve a parametro habitual.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>RESUELTA</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>Jul-2026</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Calles y Veredas</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Cancelado alto en cerrados</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>5% (sobre cerrados)</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Cancelado baja a 5% de los cerrados en Ago-2026 (donut Cierres por Estado), dentro del rango operativo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>RESUELTA</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Jul-2026</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>Transito</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>Cancelado alto en cerrados</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>8% (sobre cerrados)</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Cancelado baja a 8% de los cerrados en Ago-2026 (donut Cierres por Estado), dentro del rango operativo.</t>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>10 dias</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Tiempo promedio de resolucion 9-&gt;10 días (Ago-2026 a Sep-2026). Se mantiene elevado.</t>
         </is>
       </c>
     </row>
@@ -770,27 +770,27 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>Mar-2026</t>
+          <t>Jul-2026</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Calles y Veredas</t>
+          <t>Control de Actividades Comerciales</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>Cierre colapsado</t>
+          <t>Brecha cierre-satisfaccion</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>13%-&gt;20%</t>
+          <t>Cierre 88% / Sat 31%</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>Cierre del area 13%-&gt;20% (Jul-2026 a Ago-2026). Sigue en zona critica. Cancelado 5% sobre cerrados.</t>
+          <t>Cierre 88% con satisfaccion 31% en Sep-2026 (26 respuestas). La brecha entre gestion cerrada y percepcion del vecino se mantiene.</t>
         </is>
       </c>
     </row>
@@ -802,34 +802,34 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Jul-2026</t>
+          <t>Ago-2026</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Control de Actividades Comerciales</t>
+          <t>Control del Espacio Publico</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Brecha cierre-satisfaccion</t>
+          <t>Cierre bajo - Cable cortado</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Cierre 78% / Sat 33%</t>
+          <t>117 casos, 1% cierre</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Cierre 78% con satisfaccion 33% en Ago-2026 (tablero). La brecha entre gestion cerrada y percepcion del vecino se mantiene.</t>
+          <t>Cable cortado: 117 casos en Sep-2026 (77 en Ago-2026), cierre 12%-&gt;1%. Sigue con cierre bajo.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>NUEVA</t>
+          <t>PERSISTE</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -839,22 +839,22 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Arbolado y Plazas</t>
+          <t>Control del Espacio Publico</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>Cierre bajo (area)</t>
+          <t>Cierre bajo - Poste en mal estado/sin mantenimiento</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>49%</t>
+          <t>21 casos, 14% cierre</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>Cierre del area 49% en Ago-2026 (tablero). Cancelado 8% sobre cerrados.</t>
+          <t>Poste en mal estado/sin mantenimiento: 21 casos en Sep-2026 (24 en Ago-2026), cierre 22%-&gt;14%. Sigue con cierre bajo.</t>
         </is>
       </c>
     </row>
@@ -866,27 +866,27 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Ago-2026</t>
+          <t>Sep-2026</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Calles y Veredas</t>
+          <t>Arbolado y Plazas</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Dias promedio alto</t>
+          <t>Cancelado alto en cerrados</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>9 dias</t>
+          <t>11% (sobre cerrados)</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>Tiempo promedio de resolucion 9 dias en Ago-2026 (tablero). Por encima del tiempo habitual.</t>
+          <t>11% de los cerrados de Sep-2026 son Cancelados (8 de 74, donut Cierres por Estado): Reparación o daño de caniles en parque/plaza (5 de 7 cierres) y Inconvenientes con intervenciones de arbolado (3 de 33 cierres). Revisar la calidad de esos cierres.</t>
         </is>
       </c>
     </row>
@@ -898,27 +898,27 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Ago-2026</t>
+          <t>Sep-2026</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Control del Espacio Publico</t>
+          <t>Arbolado y Plazas</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Cierre bajo - Cable cortado</t>
+          <t>Suba de volumen - Árbol obstruye luminaria</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>12% (77 casos)</t>
+          <t>11-&gt;38 (+245%)</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>Tipo 'Cable cortado': 77 casos en Ago-2026 con 12% de cierre (tablero). Cierre muy por debajo del resto del area.</t>
+          <t>Árbol obstruye luminaria: 11 casos en Ago-2026 a 38 en Sep-2026 (+245%), maximo de los ultimos 13 meses; 11% de cierre.</t>
         </is>
       </c>
     </row>
@@ -930,27 +930,251 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Ago-2026</t>
+          <t>Sep-2026</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
+          <t>Calles y Veredas</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>SLA critico (area)</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>28%</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>SLA del area 28% en Sep-2026: 51 de los 71 cierres fuera del plazo por tipo. Tiempo promedio 10 dias.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Calles y Veredas</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Cancelado alto en cerrados</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>7% (sobre cerrados)</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>7% de los cerrados de Sep-2026 son Cancelados (5 de 71, donut Cierres por Estado): Bache en calle de asfalto (2 de 42 cierres) y Repintado / reparación de demarcación vial en calle o cordón (1 de 4 cierres). Revisar la calidad de esos cierres.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Calles y Veredas</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Suba de volumen - Reparación/construcción de cordón</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>69-&gt;111 (+61%)</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>Reparación/construcción de cordón: 69 casos en Ago-2026 a 111 en Sep-2026 (+61%), maximo de los ultimos 13 meses; 5% de cierre.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Calles y Veredas</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Suba de volumen - Reparación de rampa de accesibilidad</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>15-&gt;36 (+140%)</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>Reparación de rampa de accesibilidad: 15 casos en Ago-2026 a 36 en Sep-2026 (+140%), maximo de los ultimos 13 meses; 6% de cierre.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Calles y Veredas</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Volumen anomalo - Construcción de cuneta</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>4-&gt;22</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>Construcción de cuneta: pasa de 4 casos en Ago-2026 a 22 en Sep-2026, maximo de los ultimos 13 meses sobre una base historica baja; ningún cierre.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
           <t>Control del Espacio Publico</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>Cierre bajo - Poste en mal estado/sin mantenimiento</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>22% (23 casos)</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>Tipo 'Poste en mal estado/sin mantenimiento': 23 casos en Ago-2026 con 22% de cierre (tablero). Cierre muy por debajo del resto del area.</t>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Cierre bajo (area)</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>39%</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>Cierre del area 39% en Sep-2026 (125 de 318). Lo arrastra: Cable cortado 117 casos (1% de cierre); Reparación de vereda rota por empresa de servicio 27 casos (15% de cierre). Cancelado 2% sobre cerrados.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Control del Espacio Publico</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Suba de volumen - Reparación de vereda rota por empresa de servicio</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>19-&gt;27 (+42%)</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>Reparación de vereda rota por empresa de servicio: 19 casos en Ago-2026 a 27 en Sep-2026 (+42%), maximo de los ultimos 13 meses; 15% de cierre.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>NUEVA</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Sep-2026</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Transito</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Cancelado alto en cerrados</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>3% (sobre cerrados)</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>3% de los cerrados de Sep-2026 son Cancelados (13 de 372, donut Cierres por Estado): Vehículos Abandonados (10 de 320 cierres) y Reparación de semáforo (3 de 40 cierres). Revisar la calidad de esos cierres.</t>
         </is>
       </c>
     </row>

</xml_diff>